<commit_message>
Update result CW SW functionality
</commit_message>
<xml_diff>
--- a/frontend/public/sample_marks.xlsx
+++ b/frontend/public/sample_marks.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Marks" sheetId="1" r:id="rId1"/>
+    <sheet name="Class Marks" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,27 +397,33 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>enrollmentNo</v>
       </c>
       <c r="B1" t="str">
-        <v>internalMarks</v>
+        <v>studentName</v>
       </c>
       <c r="C1" t="str">
-        <v>externalMarks</v>
+        <v>CW (30)</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Theory (70)</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
         <v>0801IT221001</v>
       </c>
-      <c r="B2">
-        <v>35</v>
+      <c r="B2" t="str">
+        <v>Priya Nair</v>
       </c>
       <c r="C2">
+        <v>25</v>
+      </c>
+      <c r="D2">
         <v>48</v>
       </c>
     </row>
@@ -425,10 +431,13 @@
       <c r="A3" t="str">
         <v>0801IT221002</v>
       </c>
-      <c r="B3">
+      <c r="B3" t="str">
+        <v>Harsh Jain</v>
+      </c>
+      <c r="C3">
         <v>28</v>
       </c>
-      <c r="C3">
+      <c r="D3">
         <v>42</v>
       </c>
     </row>
@@ -436,16 +445,19 @@
       <c r="A4" t="str">
         <v>0801IT221003</v>
       </c>
-      <c r="B4">
-        <v>39</v>
+      <c r="B4" t="str">
+        <v>Ananya Mishra</v>
       </c>
       <c r="C4">
+        <v>29</v>
+      </c>
+      <c r="D4">
         <v>58</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>